<commit_message>
Ajustar rodízio OSID para atendimento apenas de segunda a sexta
- Recalculado sobre os 20 dias úteis do período (04-29/01/2027), não mais 26 dias corridos
- Cada dentista cobre só 2-3 dias úteis de plantão; descanso de 17-18 dias úteis (~3,4-3,6 semanas) por pessoa
- Fins de semana marcados como "sem atendimento" na escala, não contam para plantão nem descanso
- Cobertura de 1 dentista por dia útil mantida, sem furos
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013f2XRhDo2k4tpqWLL7XirX
</commit_message>
<xml_diff>
--- a/meu-projeto/Rodizio-Plantao-OSID-Jan2027.xlsx
+++ b/meu-projeto/Rodizio-Plantao-OSID-Jan2027.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,6 +41,18 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
       <sz val="10"/>
     </font>
     <font>
@@ -54,7 +66,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -79,6 +91,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -108,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -125,16 +142,19 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -517,13 +537,13 @@
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RODÍZIO DE PLANTÃO — OSID — 04 a 29/01/2027</t>
+          <t>RODÍZIO DE PLANTÃO — OSID — 04 a 29/01/2027 (atendimento seg. a sex.)</t>
         </is>
       </c>
     </row>
@@ -567,7 +587,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Início do turno</t>
+          <t>Início do plantão</t>
         </is>
       </c>
     </row>
@@ -608,80 +628,88 @@
       <c r="D5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>07/01/2027</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Quinta</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Ana Carolina Pondé</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Éder Gerardo</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Início do plantão</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>08/01/2027</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Sexta</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Éder Gerardo</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Início do turno</t>
-        </is>
-      </c>
+      <c r="D7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>09/01/2027</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Sábado</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Éder Gerardo</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr"/>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>— (sem atendimento)</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Fim de semana</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>10/01/2027</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Domingo</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Éder Gerardo</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr"/>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>— (sem atendimento)</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Fim de semana</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -719,7 +747,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Início do turno</t>
+          <t>Início do plantão</t>
         </is>
       </c>
     </row>
@@ -760,62 +788,70 @@
       <c r="D13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>15/01/2027</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Sexta</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Juliana Azevedo</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Juliana Borges</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Início do plantão</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>16/01/2027</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Sábado</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Juliana Borges</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>Início do turno</t>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>— (sem atendimento)</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Fim de semana</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>17/01/2027</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Domingo</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Juliana Borges</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr"/>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>— (sem atendimento)</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Fim de semana</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -871,7 +907,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Início do turno</t>
+          <t>Início do plantão</t>
         </is>
       </c>
     </row>
@@ -912,62 +948,70 @@
       <c r="D21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>23/01/2027</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Sábado</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Laura</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr"/>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>— (sem atendimento)</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Fim de semana</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>24/01/2027</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Domingo</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>— (sem atendimento)</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Fim de semana</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>25/01/2027</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Segunda</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>Manoela Carrera</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>Início do turno</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>25/01/2027</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Segunda</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Manoela Carrera</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Início do plantão</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -988,44 +1032,44 @@
       <c r="D25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>27/01/2027</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Quarta</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Manoela Carrera</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>28/01/2027</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Quinta</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>Tila Fortuna</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>Início do turno</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>28/01/2027</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Quinta</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Tila Fortuna</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Início do plantão</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1063,7 +1107,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
@@ -1078,223 +1122,223 @@
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Dentista</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>Dias de plantão</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Dias úteis de plantão</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Período de plantão</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>Dias de descanso</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Dias úteis de descanso</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>Período(s) de descanso</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Semanas de descanso (aprox.)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Ana Carolina Pondé</t>
         </is>
       </c>
-      <c r="B3" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>04/01 a 07/01</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>08/01 a 29/01</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="n">
-        <v>3.1</v>
+      <c r="B3" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>04/01 a 06/01</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>07/01 a 29/01</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>3.4</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Éder Gerardo</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>08/01 a 11/01</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="n">
-        <v>22</v>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>04/01 a 07/01 + 12/01 a 29/01</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="n">
-        <v>3.1</v>
+      <c r="B4" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>07/01 a 11/01</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>04/01 a 06/01 + 12/01 a 29/01</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>3.4</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Juliana Azevedo</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>12/01 a 15/01</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>04/01 a 11/01 + 16/01 a 29/01</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="n">
-        <v>3.1</v>
+      <c r="B5" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>12/01 a 14/01</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>04/01 a 11/01 + 15/01 a 29/01</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>3.4</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Juliana Borges</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>16/01 a 19/01</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="n">
-        <v>22</v>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>04/01 a 15/01 + 20/01 a 29/01</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="n">
-        <v>3.1</v>
+      <c r="B6" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>15/01 a 19/01</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>04/01 a 14/01 + 20/01 a 29/01</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>3.4</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Laura</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>20/01 a 23/01</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>04/01 a 19/01 + 24/01 a 29/01</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="n">
-        <v>3.1</v>
+      <c r="B7" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>20/01 a 22/01</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>04/01 a 19/01 + 25/01 a 29/01</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>3.4</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Manoela Carrera</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>24/01 a 26/01</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>23</v>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>04/01 a 23/01 + 27/01 a 29/01</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="n">
-        <v>3.3</v>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>25/01 a 27/01</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>04/01 a 22/01 + 28/01 a 29/01</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>3.4</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Tila Fortuna</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>27/01 a 29/01</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>04/01 a 26/01</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="n">
-        <v>3.3</v>
-      </c>
-    </row>
-    <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>Cobertura: exatamente 1 dentista de plantão por dia, sem nenhum dia de consultório vazio. Cada pessoa trabalha só 3 ou 4 dias no período inteiro — o resto (22 a 23 dias) é descanso, acima das 3 semanas (21 dias) pedidas. Em 5 dos 7 casos o descanso fica dividido em dois blocos (antes e depois do plantão); Ana Carolina Pondé e Tila Fortuna ficam com um único bloco contínuo (por estarem nas pontas do período).</t>
+      <c r="B9" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>28/01 a 29/01</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>04/01 a 27/01</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="11" ht="72" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Atendimento apenas de segunda a sexta (fins de semana fechados, não contam como dia de plantão nem de descanso). Em 20 dias úteis no período, cada dentista cobre só 2 ou 3 dias úteis de plantão — o resto (17 a 18 dias úteis, ou cerca de 3,4 a 3,6 semanas) é descanso, acima das 3 semanas pedidas. Cobertura garantida: 1 dentista de plantão em todo dia útil, sem nenhum dia de consultório vazio. Ana Carolina Pondé e Tila Fortuna ficam com descanso em bloco único (pontas do período); os demais têm o descanso dividido em dois blocos, ao redor do próprio plantão.</t>
         </is>
       </c>
     </row>

</xml_diff>